<commit_message>
Binding mechanisms ratified into the protocol; kind library reconciled to v0.2
Protocol gains the four binding mechanisms (registries as
version-bound code-consumed data; rule-to-check closure meta-test;
banned-construct planks; metamodel version in every stamp) — build
deferred with everything else. Kind library reconciled against all
rulings since drafting: R1 structural-NOT ratified (negated twins
gone), R2/R3 deferrals ratified, table_ref added, comparand-list
role retired (position owns order), IN_LIST/IN_SELECTION split
declared structural, decisions-are-lenses noted. One finding: R6
opened — 'unary' is in the library but not the doc's ratified
expression list; Sunny to rule.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_KG2_Kind_Library_TSQL_Predicates_DRAFT.xlsx
+++ b/AIVIA_Design/L1_KG2_Kind_Library_TSQL_Predicates_DRAFT.xlsx
@@ -462,7 +462,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>DRAFT v0.1 — authored by Claude 2026-09-04 as brainstorm output. Nothing ratified until Sunny lands it in the AIVIA Design Document. Scope: PREDICATE portion of the semantic grammar for T-SQL. Structure kinds (scope/FROM/JOIN/GROUP BY/UNION/CTE) and full expression grammar: own files later.</t>
+          <t>v0.2 — RECONCILED 2026-09-04 against the ratified design doc (KG Layer 2: unit, node types, edge families, 8 rules) and Sunny's rulings R1-R5. Companion of the doc's KG Layer 2 section; the doc is the authority.</t>
         </is>
       </c>
     </row>
@@ -482,7 +482,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Finite and versioned. Closed set; grows only by versioned change with a conformance case authored BEFORE the change; every stored tree is stamped with the library version.</t>
+          <t>Finite and versioned. Closed set; grows only by versioned change (doc -&gt; registry -&gt; code, never code-first) with a conformance case authored BEFORE the change.</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Totality against the vendor denominator. Every ScriptDom boolean type is mapped or deferred-with-reason, both directions, checked by reflecting the vendor enums (the spreadsheet is the readable projection; reflection is the enforcement).</t>
+          <t>Totality against the vendor denominator (reflected, never hand-typed): every vendor construct mapped or deferred-with-reason, both directions.</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>The mapper never guesses. No kind -&gt; counted remainder (reason + location + raw evidence); the rest of the file still parses.</t>
+          <t>The mapper never guesses. No kind -&gt; counted remainder (reason + location + raw evidence).</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Dialect-neutral kinds, dialect-labeled evidence. Every node carries dialect, source location, raw AST fragment. Kinds never mention T-SQL.</t>
+          <t>Dialect-neutral kinds, dialect-labeled evidence.</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Every predicate node carries: kind | site (the boolean tree at one WHERE/HAVING/JOIN-ON/CASE-WHEN/IF position) | scope owner (a derived table's filter belongs to THAT scope) | role-labeled children | evidence | version stamps.</t>
+          <t>Per the ratified doc: predicates are nodes owned by exactly one scope; role-labeled contains edges to their expression children; evidence + version stamps on every node.</t>
         </is>
       </c>
     </row>
@@ -623,12 +623,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>NOT (BooleanNotExpression); negated syntax forms per Open Ruling R1</t>
+          <t>NOT (BooleanNotExpression); ALL negated syntax forms</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>R1 recommends NOT LIKE / NOT IN / NOT BETWEEN / IS NOT NULL / NOT EXISTS normalize to NOT over the positive kind, original syntax kept in evidence.</t>
+          <t>R1 RATIFIED 2026-09-04: NOT LIKE / NOT IN / NOT BETWEEN / IS NOT NULL / NOT EXISTS normalize to NOT over the positive kind; original syntax kept in evidence. One meaning, one kind; 'all pattern-match decisions' is one graph query.</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
   </cols>
@@ -858,7 +858,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>LIKE (negation via NOT, per R1)</t>
+          <t>LIKE (negation via NOT, R1 ratified)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -876,7 +876,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>subject, comparand-list</t>
+          <t>subject, comparand (one per member, ordered by position)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Deliberately a DIFFERENT kind from IN_SELECTION: enumerated values vs delegation to data.</t>
+          <t>A DIFFERENT kind from IN_SELECTION: enumerated values vs delegation to data.</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>The clinical value-set pattern; queryable on its own.</t>
+          <t>The clinical value-set pattern; queryable on its own. Detection is STRUCTURAL (the comparand is a subquery_ref), never string-matching.</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>BETWEEN ... AND ... (BooleanTernaryExpression; negation via NOT)</t>
+          <t>BETWEEN ... AND ... (negation via NOT)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Degenerate predicates (1=1): map to their comparison kind; 'decides nothing' (both sides literal) is a DERIVED fact. CASE in predicate position: a comparison whose subject is a case-expression node. Parameter defaults (IF @p IS NULL SET @p=...): IF structure + NULL_CHECK + assignment; 'parameter default' becomes a derived pattern.</t>
+          <t>Degenerate predicates (1=1): map to their comparison kind; 'decides nothing' is a DERIVED fact (lens). CASE in predicate position: a comparison whose subject is a case expression node. Parameter defaults: IF structure + NULL_CHECK + assignment; 'parameter default' is a derived pattern. Decisions themselves: LENSES, never kinds (graph-leads ruling).</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr"/>
@@ -1034,7 +1034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1073,79 +1073,67 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>the value/expression compared against</t>
+          <t>the value/expression compared against; IN-list members are one comparand edge each, ordered by the contains edge's position property (reconciled: the former comparand-list role is retired — position owns order)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>comparand-list</t>
+          <t>lower_bound / upper_bound</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>the enumerated values of IN_LIST (order kept)</t>
+          <t>the two ends of a RANGE</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>lower_bound / upper_bound</t>
+          <t>pattern / escape</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>the two ends of a RANGE</t>
+          <t>the match pattern (and optional escape) of PATTERN_MATCH</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>pattern / escape</t>
+          <t>selection</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>the match pattern (and optional escape) of PATTERN_MATCH</t>
+          <t>a subquery scope used as the comparand (IN_SELECTION, EXISTS_SELECTION, QUANTIFIED_COMPARE) — reached via a subquery_ref child's resolves_to</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>selection</t>
+          <t>quantifier</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>a subquery scope used as the comparand (IN_SELECTION, EXISTS_SELECTION, QUANTIFIED_COMPARE)</t>
+          <t>ANY / ALL / SOME on QUANTIFIED_COMPARE</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>quantifier</t>
+          <t>(why roles)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ANY / ALL / SOME on QUANTIFIED_COMPARE</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>(why roles)</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Role labels are load-bearing: without them a predicate knows which columns participate but not what it SAYS about them — the recorded misattribution bug class (right values, wrong subject).</t>
+          <t>Role labels ride the contains edges from predicate to expression children (ratified edge design). Without them a predicate knows which columns participate but not what it SAYS about them — the recorded misattribution bug class.</t>
         </is>
       </c>
     </row>
@@ -1187,115 +1175,115 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>points at a technical-layer column node — the only cross-layer pointer</t>
+          <t>a MENTION of a column; resolves_to a KG layer 1 column node (or no edge = counted unresolved)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>literal</t>
+          <t>table_ref</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>a constant value, owned by the predicate side</t>
+          <t>a MENTION of a table; resolves_to a KG layer 1 table OR a scope in the same tree (CTE / #temp stage) — ADDED in the ratified doc (a FROM references tables)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>parameter_ref</t>
+          <t>literal</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>reference to a file-scope parameter node</t>
+          <t>a constant value, owned by the predicate side</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>function</t>
+          <t>parameter_ref</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>function application over child expressions</t>
+          <t>a mention of a parameter; resolves_to the file's parameter node</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>arithmetic</t>
+          <t>function</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>arithmetic over child expressions</t>
+          <t>function application over ordered child expressions</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>case_expr</t>
+          <t>arithmetic</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>value branching (WHENs hold predicates, THENs hold expressions)</t>
+          <t>arithmetic over child expressions</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>cast</t>
+          <t>case</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>representation change, not meaning change</t>
+          <t>value branching (WHENs hold predicates, THENs hold expressions)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>unary</t>
+          <t>cast</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>sign/negation on a value</t>
+          <t>representation change, not meaning change</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>subquery</t>
+          <t>unary</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>a nested selection used as a value</t>
+          <t>sign/negation on a value — OPEN: not yet in the ratified doc's expression list; amendment proposed (see Open_Rulings R6)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>(note)</t>
+          <t>subquery_ref</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Summary only — the full expression grammar gets its own file at the same level of detail.</t>
+          <t>a mention of a nested selection used as a value; resolves_to its scope node</t>
         </is>
       </c>
     </row>
@@ -1314,8 +1302,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1365,7 +1353,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>NOT</t>
+          <t>NOT (all negated syntax normalizes here — R1 ratified)</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1421,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>IN_LIST / IN_SELECTION</t>
+          <t>IN_LIST / IN_SELECTION (structural split: subquery_ref comparand vs literal members)</t>
         </is>
       </c>
     </row>
@@ -1530,12 +1518,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>DEFERRED (Open Ruling R2)</t>
+          <t>DEFERRED — R2 RATIFIED 2026-09-04</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>SQL 2022 null-safe equality; rare in target estates today</t>
+          <t>SQL 2022 null-safe equality; revisit on first estate sighting</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1535,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>DEFERRED (Open Ruling R3)</t>
+          <t>DEFERRED — R3 RATIFIED 2026-09-04</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1620,7 +1608,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>upstream of predicates entirely — nothing inside a runtime string is static SQL</t>
+          <t>upstream of predicates entirely</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1638,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>What is authored (BEFORE any mapper code — the answer-key law at the seam)</t>
+          <t>What is authored (BEFORE any mapper code — protocol step 4)</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1662,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>the recorded corpse catalog: OR shapes, derived-table scope, RANGE over columns, IN_SELECTION value sets, CTE referenced twice, 1=1, CASE-in-predicate</t>
+          <t>the recorded corpse catalog: OR shapes, derived-table scope, RANGE over columns, IN_SELECTION value sets, CTE referenced twice, 1=1, CASE-in-predicate, temp-table staging chains, negated forms (R1), nested control-flow statements</t>
         </is>
       </c>
     </row>
@@ -1713,12 +1701,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="66" customWidth="1" min="2" max="2"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1734,7 +1722,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Recommendation</t>
+          <t>Status</t>
         </is>
       </c>
     </row>
@@ -1746,12 +1734,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Negation: normalize NOT LIKE / NOT IN / NOT BETWEEN / IS NOT NULL / NOT EXISTS to structural NOT over the positive kind, or keep negated twin kinds matching the AST flags (today's code)?</t>
+          <t>Negation normalization</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Normalize to NOT; one meaning one kind; 'all pattern-match decisions' stays one graph query; syntax kept in evidence</t>
+          <t>RATIFIED 2026-09-04: structural NOT over the positive kind; syntax in evidence</t>
         </is>
       </c>
     </row>
@@ -1763,12 +1751,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>IS [NOT] DISTINCT FROM: defer or admit NULL_SAFE_EQ kind?</t>
+          <t>IS [NOT] DISTINCT FROM</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Defer for now, revisit on first estate sighting</t>
+          <t>RATIFIED 2026-09-04: deferred; revisit on first estate sighting</t>
         </is>
       </c>
     </row>
@@ -1780,12 +1768,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Full-text predicates: defer or admit TEXT_SEARCH kind?</t>
+          <t>Full-text predicates</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Defer</t>
+          <t>RATIFIED 2026-09-04: deferred</t>
         </is>
       </c>
     </row>
@@ -1797,12 +1785,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>The word for derived readings of the graph ('view' is poisoned): lens? facet?</t>
+          <t>'lens' for derived readings</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>lens</t>
+          <t>RATIFIED (landed in the doc's Level 0)</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1802,29 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>The word for the kind/role/rule layer ('schema' -&gt; ?)</t>
+          <t>'metamodel' for the kind/role/rule layer</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>metamodel (Collibra's own term for exactly this; Purview equivalent = its type system)</t>
+          <t>RATIFIED (in use throughout the doc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>unary expression kind: in this library but NOT in the ratified doc's expression list — add 'unary' to the doc, or fold sign-negation into arithmetic?</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — found during reconciliation; Sunny to rule</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
R6 ratified: unary in the doc's expression list; workbook closed to match
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_KG2_Kind_Library_TSQL_Predicates_DRAFT.xlsx
+++ b/AIVIA_Design/L1_KG2_Kind_Library_TSQL_Predicates_DRAFT.xlsx
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>sign/negation on a value — OPEN: not yet in the ratified doc's expression list; amendment proposed (see Open_Rulings R6)</t>
+          <t>sign/negation on a value (in the ratified doc list — R6 ratified 2026-09-04)</t>
         </is>
       </c>
     </row>
@@ -1824,7 +1824,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>OPEN — found during reconciliation; Sunny to rule</t>
+          <t>RATIFIED 2026-09-04: 'unary' added to the doc's expression list</t>
         </is>
       </c>
     </row>

</xml_diff>